<commit_message>
build: Cập nhật dữ liệu và giao diện Online 24/24
</commit_message>
<xml_diff>
--- a/03.QLDA/A320.xlsx
+++ b/03.QLDA/A320.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AMECC JSC\Amecc 2\00. Overall Report\03.QLDA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14B3B6A-C7ED-497F-8BB5-0F6EA241BB57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9C2FBCF-67E6-4EB3-A1E6-5D6B685C3BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EB65E7D8-5C33-4F00-97F9-F6CAD846FF50}"/>
   </bookViews>
@@ -55,9 +55,9 @@
     <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" hidden="1">#REF!</definedName>
     <definedName name="ㅌㅊㅍㅌㅊㅍㅌㅋㅊㅍㅌ" hidden="1">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1"/>
   <pivotCaches>
-    <pivotCache cacheId="40" r:id="rId2"/>
+    <pivotCache cacheId="93" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1893" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1896" uniqueCount="277">
   <si>
     <t>Gá lắp</t>
   </si>
@@ -905,6 +905,12 @@
   <si>
     <t>A320-001</t>
   </si>
+  <si>
+    <t>A320-002</t>
+  </si>
+  <si>
+    <t>A320-M4130-006</t>
+  </si>
 </sst>
 </file>
 
@@ -1603,7 +1609,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="DELL" refreshedDate="46282.457814236113" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="323" xr:uid="{4067F58C-28E2-44CB-8FA2-A8EFFD878FFB}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="DELL" refreshedDate="46293.337688425927" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="323" xr:uid="{4067F58C-28E2-44CB-8FA2-A8EFFD878FFB}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A3:BA326" sheet="Progress"/>
   </cacheSource>
@@ -1771,19 +1777,19 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0" maxValue="6461.7199999999975"/>
     </cacheField>
     <cacheField name="Ngày BG" numFmtId="14">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="2026-09-16T00:00:00" maxDate="2026-09-24T00:00:00"/>
     </cacheField>
     <cacheField name="SL BG" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="1"/>
     </cacheField>
     <cacheField name="KL BG" numFmtId="43">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="0"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0" maxValue="6461.7199999999975"/>
     </cacheField>
     <cacheField name="Đơn vị nhận" numFmtId="0">
       <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="Số biên bản" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -10095,11 +10101,11 @@
     <d v="2026-09-16T00:00:00"/>
     <n v="1"/>
     <n v="2369"/>
-    <m/>
-    <m/>
-    <n v="0"/>
+    <d v="2026-09-23T00:00:00"/>
+    <n v="1"/>
+    <n v="2369"/>
     <s v="PAC"/>
-    <m/>
+    <s v="A320-002"/>
   </r>
   <r>
     <n v="152"/>
@@ -10150,11 +10156,11 @@
     <d v="2026-09-16T00:00:00"/>
     <n v="1"/>
     <n v="2397.3999999999996"/>
-    <m/>
-    <m/>
-    <n v="0"/>
+    <d v="2026-09-23T00:00:00"/>
+    <n v="1"/>
+    <n v="2397.3999999999996"/>
     <s v="PAC"/>
-    <m/>
+    <s v="A320-002"/>
   </r>
   <r>
     <n v="153"/>
@@ -10205,11 +10211,11 @@
     <d v="2026-09-11T00:00:00"/>
     <n v="1"/>
     <n v="6461.7199999999975"/>
-    <m/>
-    <m/>
-    <n v="0"/>
+    <d v="2026-09-16T00:00:00"/>
+    <n v="1"/>
+    <n v="6461.7199999999975"/>
     <s v="PAC"/>
-    <m/>
+    <s v="A320-001"/>
   </r>
   <r>
     <n v="154"/>
@@ -10260,11 +10266,11 @@
     <d v="2026-09-11T00:00:00"/>
     <n v="1"/>
     <n v="5173.1000000000004"/>
-    <m/>
-    <m/>
-    <n v="0"/>
+    <d v="2026-09-16T00:00:00"/>
+    <n v="1"/>
+    <n v="5173.1000000000004"/>
     <s v="PAC"/>
-    <m/>
+    <s v="A320-001"/>
   </r>
   <r>
     <n v="155"/>
@@ -10315,11 +10321,11 @@
     <d v="2026-09-11T00:00:00"/>
     <n v="1"/>
     <n v="4180.7848000000004"/>
-    <m/>
-    <m/>
-    <n v="0"/>
+    <d v="2026-09-16T00:00:00"/>
+    <n v="1"/>
+    <n v="4180.7848000000004"/>
     <s v="PAC"/>
-    <m/>
+    <s v="A320-001"/>
   </r>
   <r>
     <n v="156"/>
@@ -19565,7 +19571,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85CD8DED-1024-4DD7-B7B9-B699E3BC5DA2}" name="PivotTable2" cacheId="40" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85CD8DED-1024-4DD7-B7B9-B699E3BC5DA2}" name="PivotTable2" cacheId="93" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="BF3:BH13" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="53">
     <pivotField showAll="0"/>
@@ -20396,7 +20402,7 @@
       <c r="R2" s="5"/>
       <c r="S2" s="51">
         <f ca="1">IF(WEEKDAY(TODAY()-1)=1,TODAY()-2,TODAY()-1)</f>
-        <v>46281</v>
+        <v>46291</v>
       </c>
       <c r="T2" s="13" t="s">
         <v>40</v>
@@ -20452,20 +20458,20 @@
       <c r="AT2" s="17"/>
       <c r="AU2" s="67">
         <f>SUBTOTAL(9,AU4:AU326)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AV2" s="68">
         <f>SUBTOTAL(9,AV4:AV326)</f>
-        <v>20582.004799999999</v>
+        <v>22652.604800000001</v>
       </c>
       <c r="AW2" s="16"/>
       <c r="AX2" s="67">
         <f>SUBTOTAL(9,AX4:AX326)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AY2" s="67">
         <f>SUBTOTAL(9,AY4:AY326)</f>
-        <v>15815.604799999997</v>
+        <v>20582.004799999999</v>
       </c>
       <c r="AZ2" s="17"/>
       <c r="BA2" s="18" t="str">
@@ -36878,11 +36884,11 @@
       <c r="AD143" s="54"/>
       <c r="AE143" s="31">
         <f t="shared" si="29"/>
-        <v>1863.54</v>
+        <v>2070.6</v>
       </c>
       <c r="AF143" s="32">
         <f t="shared" si="30"/>
-        <v>207.05999999999995</v>
+        <v>0</v>
       </c>
       <c r="AG143" s="30"/>
       <c r="AH143" s="33">
@@ -36918,12 +36924,18 @@
         <f t="shared" si="34"/>
         <v>0</v>
       </c>
-      <c r="AS143" s="27"/>
-      <c r="AT143" s="37"/>
-      <c r="AU143" s="30"/>
+      <c r="AS143" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="AT143" s="37">
+        <v>46291</v>
+      </c>
+      <c r="AU143" s="30">
+        <v>1</v>
+      </c>
       <c r="AV143" s="36">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>2070.6</v>
       </c>
       <c r="AW143" s="35"/>
       <c r="AX143" s="30"/>
@@ -38317,16 +38329,22 @@
         <f t="shared" si="35"/>
         <v>2369</v>
       </c>
-      <c r="AW154" s="35"/>
-      <c r="AX154" s="30"/>
+      <c r="AW154" s="35">
+        <v>46288</v>
+      </c>
+      <c r="AX154" s="30">
+        <v>1</v>
+      </c>
       <c r="AY154" s="32">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>2369</v>
       </c>
       <c r="AZ154" s="30" t="s">
         <v>265</v>
       </c>
-      <c r="BA154" s="63"/>
+      <c r="BA154" s="63" t="s">
+        <v>275</v>
+      </c>
       <c r="BB154" s="71"/>
       <c r="BC154" s="71"/>
       <c r="BD154" s="71"/>
@@ -38449,16 +38467,22 @@
         <f t="shared" si="35"/>
         <v>2397.3999999999996</v>
       </c>
-      <c r="AW155" s="35"/>
-      <c r="AX155" s="30"/>
+      <c r="AW155" s="35">
+        <v>46288</v>
+      </c>
+      <c r="AX155" s="30">
+        <v>1</v>
+      </c>
       <c r="AY155" s="32">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>2397.3999999999996</v>
       </c>
       <c r="AZ155" s="30" t="s">
         <v>265</v>
       </c>
-      <c r="BA155" s="63"/>
+      <c r="BA155" s="63" t="s">
+        <v>275</v>
+      </c>
       <c r="BB155" s="71"/>
       <c r="BC155" s="71"/>
       <c r="BD155" s="71"/>

</xml_diff>